<commit_message>
RTM v0.10: NFR-3.5 test case and execution evidence state each secret scan's scope
O70 and Q70: the PR scan covers the full history of the PR's merge result (HEAD --full-history) plus the extracted Office text; the weekly scan covers all branches. P70 unchanged (AC-NFR-3.5's wording). Raised in review by C. Burger.
</commit_message>
<xml_diff>
--- a/docs/Requirements/Requirements Traceability Matrix/Requirements_Traceability_Matrix_v0.10.xlsx
+++ b/docs/Requirements/Requirements Traceability Matrix/Requirements_Traceability_Matrix_v0.10.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4c906530d9ff38bc/Desktop/SEN381/Ticketing-System/docs/Requirements/Requirements Traceability Matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="13_ncr:1_{B985FB7A-2EB4-42A8-80CA-EA96F303AA9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F3075BA6-508C-41BA-A1E8-C0B9BA589AD1}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="13_ncr:1_{B985FB7A-2EB4-42A8-80CA-EA96F303AA9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B39FE5B2-4D76-4EA0-9995-D8807106810A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2212,15 +2212,9 @@
     <t>Implemented. No open defect</t>
   </si>
   <si>
-    <t>CI secret scan (Gitleaks, full history) on every PR; weekly all-branch scan</t>
-  </si>
-  <si>
     <t>From AC-NFR-3.5: a secret scan of the full history reports no password, key, token or connection secret</t>
   </si>
   <si>
-    <t>Every CI run, including 38737312900 (v3.0-M3-rc tree); all-branch run 38735993793 (15/10/2026): no leaks</t>
-  </si>
-  <si>
     <t>Implemented. Six reviewed false positives ignored by fingerprint (.gitleaksignore). No open defect</t>
   </si>
   <si>
@@ -2261,6 +2255,12 @@
   </si>
   <si>
     <t>Live artefact, version 0.9 at Milestone 3. Source, requirement and acceptance criteria were populated at M1. The ASR, architecture, data, design, technology, implementation and verification columns were introduced at M2: populated where M2 evidence exists, and carried at a controlled status where it legitimately does not. v0.5 (29/09/2026, R. van der Merwe): data/persistence column completed for all 79 rows; DEC-015 to DEC-017 and CR-001 to CR-004 referenced. Change notes: RTM_v0.5_Change_Notes.md. v0.6 (30/09/2026, C. Burger): ASR / quality-driver link and Architecture / module / component columns completed for all 79 rows from PED §6A (ASR-01 to ASR-06, DEC-014); requirements with no driver are marked explicitly. v0.7 (30/09/2026, R. van der Merwe): Implementation and Verification evidence populated for the 11 requirements the application slice now implements (FR-1.3, FR-1.5, FR-2.2, FR-3.5, FR-6.1 to FR-6.7), after PR #63; FR-1.5, FR-2.2 and FR-3.5 are recorded as partial. Status column unchanged. v0.8 (30/09/2026, E. Lindsay): NFR-3.3 Implementation and Verification evidence added; FR-1.3 and FR-6.7 corrected from Implemented to Partially implemented (AC-FR-1.3 rejected-attempt recording not built; DB-01 layer 3 is M3). Status column unchanged. v0.9 (11/10/2026, E. Lindsay): Implementation and Verification evidence added for FR-1.1, FR-1.4, NFR-1.4, NFR-1.6 and NFR-3.4 after the M3 Phase 0 composition root (PR #83, DEC-018); FR-1.1, FR-1.4 and NFR-1.4 recorded as partial. Design / interface entries for DEC-018 added on the same five rows. The application is reachable over HTTP against the Atlas test cluster (SMOKE-01); no index is evidenced on the cluster. Status column unchanged. Also corrected in v0.9: the NFR-3.4 Data/persistence cell, which said the TTL index enforces idle expiry — DB-01 v0.3 §3.9 states that reading is wrong, and the enforcement is in the application against lastSeenAt (R. van der Merwe's column, corrected by E. Lindsay and notified). The Architecture column on FR-1.4, NFR-1.6 and NFR-3.4 changed from "(planned)" to reflect the composed application (C. Burger's column, corrected by E. Lindsay and notified). NOTE ON EVIDENCE: Implementation and verification evidence is recorded at component level. Each component named is implemented and verified by npm test, with its collaborators substituted (no database, no HTTP). Since v0.9 the composition root (src/composition.js, src/server.js) composes the routes, services, repositories and unit of work, and the session middleware sets req.actor; the application is reachable over HTTP against the Atlas test cluster, recorded in docs/evidence/M3-P0/SMOKE-01_phase0_reachability.txt. SMOKE-01 is reachability evidence only: it does not show that any index exists on the cluster. Where a row cites SMOKE-01, that check ran against the cluster; every other cited test ran without a database. Verification that needs a live database (transaction atomicity and rollback, DB-01 layer 3, audit-trigger lag) is M3. v0.10 (15/10/2026, E. Lindsay): the M3 chain added as four columns (O test cases, P expected result, Q execution evidence, R defect / M3 status), populated for the 27 requirements the M3 release candidate (v3.0-M3-rc) implements or verifies; the other 52 rows are marked "Not in M3 scope" with the reason. Unit evidence is the CI run at the release candidate (Node 22); test evidence records UT-1 to UT-5 and BB-1 to BB-5 (M3_Test_Evidence_Records_v0.1.md); API cases on the test cluster; E2E at v3.0-M3-rc; staging, NFR-2.4 and smoke from the staging deploy record. Defects and debt cited: DEF-011, DEF-019, DEF-020, TD-005, TD-006, TD-008; open items OI-01, OI-15, OI-16, OI-17, OI-18. Columns A to N and the Status summary sheet unchanged.</t>
+  </si>
+  <si>
+    <t>Gitleaks on every PR over the full history of the PR's merge result (--log-opts "HEAD --full-history"), plus the extracted text of every committed version of every Office document; weekly full-history scan of all branches (secret-scan-all-branches.yml)</t>
+  </si>
+  <si>
+    <t>Every CI run, including 38737312900 (v3.0-M3-rc tree): no leaks in the history of HEAD or the Office text; all-branch run 38735993793 (15/10/2026): no leaks</t>
   </si>
 </sst>
 </file>
@@ -2427,16 +2427,16 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2770,40 +2770,40 @@
       </c>
     </row>
     <row r="2" spans="1:18" ht="111.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="17" t="s">
-        <v>740</v>
-      </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="17"/>
-      <c r="L2" s="17"/>
-      <c r="M2" s="17"/>
-      <c r="N2" s="17"/>
+      <c r="A2" s="19" t="s">
+        <v>738</v>
+      </c>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="19"/>
+      <c r="L2" s="19"/>
+      <c r="M2" s="19"/>
+      <c r="N2" s="19"/>
     </row>
     <row r="3" spans="1:18" ht="70.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="16"/>
-      <c r="J3" s="16"/>
-      <c r="K3" s="16"/>
-      <c r="L3" s="16"/>
-      <c r="M3" s="16"/>
-      <c r="N3" s="16"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
+      <c r="M3" s="18"/>
+      <c r="N3" s="18"/>
     </row>
     <row r="5" spans="1:18" ht="24" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -2848,16 +2848,16 @@
       <c r="N5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="O5" s="18" t="s">
+      <c r="O5" s="15" t="s">
         <v>628</v>
       </c>
-      <c r="P5" s="18" t="s">
+      <c r="P5" s="15" t="s">
         <v>629</v>
       </c>
-      <c r="Q5" s="18" t="s">
+      <c r="Q5" s="15" t="s">
         <v>630</v>
       </c>
-      <c r="R5" s="18" t="s">
+      <c r="R5" s="15" t="s">
         <v>631</v>
       </c>
     </row>
@@ -2904,16 +2904,16 @@
       <c r="N6" s="4" t="s">
         <v>600</v>
       </c>
-      <c r="O6" s="19" t="s">
+      <c r="O6" s="16" t="s">
         <v>632</v>
       </c>
-      <c r="P6" s="19" t="s">
+      <c r="P6" s="16" t="s">
         <v>633</v>
       </c>
-      <c r="Q6" s="19" t="s">
+      <c r="Q6" s="16" t="s">
         <v>634</v>
       </c>
-      <c r="R6" s="19" t="s">
+      <c r="R6" s="16" t="s">
         <v>635</v>
       </c>
     </row>
@@ -2960,16 +2960,16 @@
       <c r="N7" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="O7" s="19" t="s">
+      <c r="O7" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P7" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q7" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R7" s="19" t="s">
+      <c r="P7" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q7" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R7" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -3016,16 +3016,16 @@
       <c r="N8" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="O8" s="19" t="s">
+      <c r="O8" s="16" t="s">
         <v>638</v>
       </c>
-      <c r="P8" s="19" t="s">
+      <c r="P8" s="16" t="s">
         <v>639</v>
       </c>
-      <c r="Q8" s="19" t="s">
+      <c r="Q8" s="16" t="s">
         <v>640</v>
       </c>
-      <c r="R8" s="19" t="s">
+      <c r="R8" s="16" t="s">
         <v>641</v>
       </c>
     </row>
@@ -3072,16 +3072,16 @@
       <c r="N9" s="4" t="s">
         <v>605</v>
       </c>
-      <c r="O9" s="19" t="s">
+      <c r="O9" s="16" t="s">
         <v>642</v>
       </c>
-      <c r="P9" s="19" t="s">
+      <c r="P9" s="16" t="s">
         <v>643</v>
       </c>
-      <c r="Q9" s="19" t="s">
+      <c r="Q9" s="16" t="s">
         <v>644</v>
       </c>
-      <c r="R9" s="19" t="s">
+      <c r="R9" s="16" t="s">
         <v>645</v>
       </c>
     </row>
@@ -3128,16 +3128,16 @@
       <c r="N10" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="O10" s="19" t="s">
+      <c r="O10" s="16" t="s">
         <v>646</v>
       </c>
-      <c r="P10" s="19" t="s">
+      <c r="P10" s="16" t="s">
         <v>647</v>
       </c>
-      <c r="Q10" s="19" t="s">
+      <c r="Q10" s="16" t="s">
         <v>648</v>
       </c>
-      <c r="R10" s="19" t="s">
+      <c r="R10" s="16" t="s">
         <v>649</v>
       </c>
     </row>
@@ -3184,16 +3184,16 @@
       <c r="N11" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="O11" s="19" t="s">
+      <c r="O11" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P11" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q11" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R11" s="19" t="s">
+      <c r="P11" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q11" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R11" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -3240,16 +3240,16 @@
       <c r="N12" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="O12" s="19" t="s">
+      <c r="O12" s="16" t="s">
         <v>650</v>
       </c>
-      <c r="P12" s="19" t="s">
+      <c r="P12" s="16" t="s">
         <v>651</v>
       </c>
-      <c r="Q12" s="19" t="s">
+      <c r="Q12" s="16" t="s">
         <v>644</v>
       </c>
-      <c r="R12" s="19" t="s">
+      <c r="R12" s="16" t="s">
         <v>652</v>
       </c>
     </row>
@@ -3296,16 +3296,16 @@
       <c r="N13" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="O13" s="19" t="s">
+      <c r="O13" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P13" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q13" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R13" s="19" t="s">
+      <c r="P13" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q13" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R13" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -3352,16 +3352,16 @@
       <c r="N14" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="O14" s="19" t="s">
+      <c r="O14" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P14" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q14" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R14" s="19" t="s">
+      <c r="P14" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q14" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R14" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -3408,16 +3408,16 @@
       <c r="N15" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="O15" s="19" t="s">
+      <c r="O15" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P15" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q15" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R15" s="19" t="s">
+      <c r="P15" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q15" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R15" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -3464,16 +3464,16 @@
       <c r="N16" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="O16" s="19" t="s">
+      <c r="O16" s="16" t="s">
         <v>653</v>
       </c>
-      <c r="P16" s="19" t="s">
+      <c r="P16" s="16" t="s">
         <v>654</v>
       </c>
-      <c r="Q16" s="19" t="s">
+      <c r="Q16" s="16" t="s">
         <v>655</v>
       </c>
-      <c r="R16" s="19" t="s">
+      <c r="R16" s="16" t="s">
         <v>656</v>
       </c>
     </row>
@@ -3520,16 +3520,16 @@
       <c r="N17" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="O17" s="19" t="s">
+      <c r="O17" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P17" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q17" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R17" s="19" t="s">
+      <c r="P17" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q17" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R17" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -3576,16 +3576,16 @@
       <c r="N18" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="O18" s="19" t="s">
+      <c r="O18" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P18" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q18" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R18" s="19" t="s">
+      <c r="P18" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q18" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R18" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -3632,16 +3632,16 @@
       <c r="N19" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="O19" s="19" t="s">
+      <c r="O19" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P19" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q19" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R19" s="19" t="s">
+      <c r="P19" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q19" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R19" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -3688,16 +3688,16 @@
       <c r="N20" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="O20" s="19" t="s">
+      <c r="O20" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P20" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q20" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R20" s="19" t="s">
+      <c r="P20" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q20" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R20" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -3744,16 +3744,16 @@
       <c r="N21" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="O21" s="19" t="s">
+      <c r="O21" s="16" t="s">
         <v>657</v>
       </c>
-      <c r="P21" s="19" t="s">
+      <c r="P21" s="16" t="s">
         <v>658</v>
       </c>
-      <c r="Q21" s="19" t="s">
+      <c r="Q21" s="16" t="s">
         <v>659</v>
       </c>
-      <c r="R21" s="19" t="s">
+      <c r="R21" s="16" t="s">
         <v>660</v>
       </c>
     </row>
@@ -3800,16 +3800,16 @@
       <c r="N22" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="O22" s="19" t="s">
+      <c r="O22" s="16" t="s">
         <v>661</v>
       </c>
-      <c r="P22" s="19" t="s">
+      <c r="P22" s="16" t="s">
         <v>662</v>
       </c>
-      <c r="Q22" s="19" t="s">
+      <c r="Q22" s="16" t="s">
         <v>663</v>
       </c>
-      <c r="R22" s="19" t="s">
+      <c r="R22" s="16" t="s">
         <v>664</v>
       </c>
     </row>
@@ -3856,16 +3856,16 @@
       <c r="N23" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="O23" s="19" t="s">
+      <c r="O23" s="16" t="s">
         <v>665</v>
       </c>
-      <c r="P23" s="19" t="s">
+      <c r="P23" s="16" t="s">
         <v>666</v>
       </c>
-      <c r="Q23" s="19" t="s">
+      <c r="Q23" s="16" t="s">
         <v>667</v>
       </c>
-      <c r="R23" s="19" t="s">
+      <c r="R23" s="16" t="s">
         <v>668</v>
       </c>
     </row>
@@ -3912,16 +3912,16 @@
       <c r="N24" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="O24" s="19" t="s">
+      <c r="O24" s="16" t="s">
         <v>669</v>
       </c>
-      <c r="P24" s="19" t="s">
+      <c r="P24" s="16" t="s">
         <v>670</v>
       </c>
-      <c r="Q24" s="19" t="s">
+      <c r="Q24" s="16" t="s">
         <v>671</v>
       </c>
-      <c r="R24" s="19" t="s">
+      <c r="R24" s="16" t="s">
         <v>672</v>
       </c>
     </row>
@@ -3968,16 +3968,16 @@
       <c r="N25" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="O25" s="19" t="s">
+      <c r="O25" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P25" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q25" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R25" s="19" t="s">
+      <c r="P25" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q25" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R25" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -4024,16 +4024,16 @@
       <c r="N26" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="O26" s="19" t="s">
+      <c r="O26" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P26" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q26" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R26" s="19" t="s">
+      <c r="P26" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q26" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R26" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -4080,16 +4080,16 @@
       <c r="N27" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="O27" s="19" t="s">
+      <c r="O27" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P27" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q27" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R27" s="19" t="s">
+      <c r="P27" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q27" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R27" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -4136,16 +4136,16 @@
       <c r="N28" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="O28" s="19" t="s">
+      <c r="O28" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P28" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q28" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R28" s="19" t="s">
+      <c r="P28" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q28" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R28" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -4192,16 +4192,16 @@
       <c r="N29" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="O29" s="19" t="s">
+      <c r="O29" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P29" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q29" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R29" s="19" t="s">
+      <c r="P29" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q29" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R29" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -4248,16 +4248,16 @@
       <c r="N30" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="O30" s="19" t="s">
+      <c r="O30" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P30" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q30" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R30" s="19" t="s">
+      <c r="P30" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q30" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R30" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -4304,16 +4304,16 @@
       <c r="N31" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="O31" s="19" t="s">
+      <c r="O31" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P31" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q31" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R31" s="19" t="s">
+      <c r="P31" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q31" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R31" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -4360,16 +4360,16 @@
       <c r="N32" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="O32" s="19" t="s">
+      <c r="O32" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P32" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q32" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R32" s="19" t="s">
+      <c r="P32" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q32" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R32" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -4416,16 +4416,16 @@
       <c r="N33" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="O33" s="19" t="s">
+      <c r="O33" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P33" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q33" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R33" s="19" t="s">
+      <c r="P33" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q33" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R33" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -4472,16 +4472,16 @@
       <c r="N34" s="4" t="s">
         <v>235</v>
       </c>
-      <c r="O34" s="19" t="s">
+      <c r="O34" s="16" t="s">
         <v>673</v>
       </c>
-      <c r="P34" s="19" t="s">
+      <c r="P34" s="16" t="s">
         <v>674</v>
       </c>
-      <c r="Q34" s="19" t="s">
+      <c r="Q34" s="16" t="s">
         <v>675</v>
       </c>
-      <c r="R34" s="19" t="s">
+      <c r="R34" s="16" t="s">
         <v>676</v>
       </c>
     </row>
@@ -4528,16 +4528,16 @@
       <c r="N35" s="4" t="s">
         <v>245</v>
       </c>
-      <c r="O35" s="19" t="s">
+      <c r="O35" s="16" t="s">
         <v>677</v>
       </c>
-      <c r="P35" s="19" t="s">
+      <c r="P35" s="16" t="s">
         <v>678</v>
       </c>
-      <c r="Q35" s="19" t="s">
+      <c r="Q35" s="16" t="s">
         <v>679</v>
       </c>
-      <c r="R35" s="19" t="s">
+      <c r="R35" s="16" t="s">
         <v>680</v>
       </c>
     </row>
@@ -4584,16 +4584,16 @@
       <c r="N36" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="O36" s="19" t="s">
+      <c r="O36" s="16" t="s">
         <v>681</v>
       </c>
-      <c r="P36" s="19" t="s">
+      <c r="P36" s="16" t="s">
         <v>682</v>
       </c>
-      <c r="Q36" s="19" t="s">
+      <c r="Q36" s="16" t="s">
         <v>683</v>
       </c>
-      <c r="R36" s="19" t="s">
+      <c r="R36" s="16" t="s">
         <v>684</v>
       </c>
     </row>
@@ -4640,16 +4640,16 @@
       <c r="N37" s="4" t="s">
         <v>261</v>
       </c>
-      <c r="O37" s="19" t="s">
+      <c r="O37" s="16" t="s">
         <v>685</v>
       </c>
-      <c r="P37" s="19" t="s">
+      <c r="P37" s="16" t="s">
         <v>686</v>
       </c>
-      <c r="Q37" s="19" t="s">
+      <c r="Q37" s="16" t="s">
         <v>687</v>
       </c>
-      <c r="R37" s="19" t="s">
+      <c r="R37" s="16" t="s">
         <v>688</v>
       </c>
     </row>
@@ -4696,16 +4696,16 @@
       <c r="N38" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="O38" s="19" t="s">
+      <c r="O38" s="16" t="s">
         <v>689</v>
       </c>
-      <c r="P38" s="19" t="s">
+      <c r="P38" s="16" t="s">
         <v>690</v>
       </c>
-      <c r="Q38" s="19" t="s">
+      <c r="Q38" s="16" t="s">
         <v>691</v>
       </c>
-      <c r="R38" s="19" t="s">
+      <c r="R38" s="16" t="s">
         <v>692</v>
       </c>
     </row>
@@ -4752,16 +4752,16 @@
       <c r="N39" s="4" t="s">
         <v>279</v>
       </c>
-      <c r="O39" s="19" t="s">
+      <c r="O39" s="16" t="s">
         <v>693</v>
       </c>
-      <c r="P39" s="19" t="s">
+      <c r="P39" s="16" t="s">
         <v>694</v>
       </c>
-      <c r="Q39" s="19" t="s">
+      <c r="Q39" s="16" t="s">
         <v>695</v>
       </c>
-      <c r="R39" s="19" t="s">
+      <c r="R39" s="16" t="s">
         <v>696</v>
       </c>
     </row>
@@ -4808,16 +4808,16 @@
       <c r="N40" s="4" t="s">
         <v>287</v>
       </c>
-      <c r="O40" s="19" t="s">
+      <c r="O40" s="16" t="s">
         <v>697</v>
       </c>
-      <c r="P40" s="19" t="s">
+      <c r="P40" s="16" t="s">
         <v>698</v>
       </c>
-      <c r="Q40" s="19" t="s">
+      <c r="Q40" s="16" t="s">
         <v>699</v>
       </c>
-      <c r="R40" s="19" t="s">
+      <c r="R40" s="16" t="s">
         <v>700</v>
       </c>
     </row>
@@ -4864,16 +4864,16 @@
       <c r="N41" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="O41" s="19" t="s">
+      <c r="O41" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P41" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q41" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R41" s="19" t="s">
+      <c r="P41" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q41" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R41" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -4920,16 +4920,16 @@
       <c r="N42" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="O42" s="19" t="s">
+      <c r="O42" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P42" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q42" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R42" s="19" t="s">
+      <c r="P42" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q42" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R42" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -4976,16 +4976,16 @@
       <c r="N43" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="O43" s="19" t="s">
+      <c r="O43" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P43" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q43" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R43" s="19" t="s">
+      <c r="P43" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q43" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R43" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -5032,16 +5032,16 @@
       <c r="N44" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="O44" s="19" t="s">
+      <c r="O44" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P44" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q44" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R44" s="19" t="s">
+      <c r="P44" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q44" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R44" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -5088,16 +5088,16 @@
       <c r="N45" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="O45" s="19" t="s">
+      <c r="O45" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P45" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q45" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R45" s="19" t="s">
+      <c r="P45" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q45" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R45" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -5144,16 +5144,16 @@
       <c r="N46" s="4" t="s">
         <v>324</v>
       </c>
-      <c r="O46" s="19" t="s">
+      <c r="O46" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P46" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q46" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R46" s="19" t="s">
+      <c r="P46" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q46" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R46" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -5200,16 +5200,16 @@
       <c r="N47" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="O47" s="19" t="s">
+      <c r="O47" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P47" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q47" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R47" s="19" t="s">
+      <c r="P47" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q47" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R47" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -5256,16 +5256,16 @@
       <c r="N48" s="4" t="s">
         <v>334</v>
       </c>
-      <c r="O48" s="19" t="s">
+      <c r="O48" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P48" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q48" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R48" s="19" t="s">
+      <c r="P48" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q48" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R48" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -5312,16 +5312,16 @@
       <c r="N49" s="4" t="s">
         <v>341</v>
       </c>
-      <c r="O49" s="19" t="s">
+      <c r="O49" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P49" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q49" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R49" s="19" t="s">
+      <c r="P49" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q49" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R49" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -5368,16 +5368,16 @@
       <c r="N50" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="O50" s="19" t="s">
+      <c r="O50" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P50" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q50" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R50" s="19" t="s">
+      <c r="P50" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q50" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R50" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -5424,16 +5424,16 @@
       <c r="N51" s="4" t="s">
         <v>353</v>
       </c>
-      <c r="O51" s="19" t="s">
+      <c r="O51" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P51" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q51" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R51" s="19" t="s">
+      <c r="P51" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q51" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R51" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -5480,16 +5480,16 @@
       <c r="N52" s="4" t="s">
         <v>361</v>
       </c>
-      <c r="O52" s="19" t="s">
+      <c r="O52" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P52" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q52" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R52" s="19" t="s">
+      <c r="P52" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q52" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R52" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -5536,16 +5536,16 @@
       <c r="N53" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="O53" s="19" t="s">
+      <c r="O53" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P53" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q53" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R53" s="19" t="s">
+      <c r="P53" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q53" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R53" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -5592,16 +5592,16 @@
       <c r="N54" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="O54" s="19" t="s">
+      <c r="O54" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P54" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q54" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R54" s="19" t="s">
+      <c r="P54" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q54" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R54" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -5648,16 +5648,16 @@
       <c r="N55" s="4" t="s">
         <v>383</v>
       </c>
-      <c r="O55" s="19" t="s">
+      <c r="O55" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P55" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q55" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R55" s="19" t="s">
+      <c r="P55" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q55" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R55" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -5704,16 +5704,16 @@
       <c r="N56" s="4" t="s">
         <v>391</v>
       </c>
-      <c r="O56" s="19" t="s">
+      <c r="O56" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P56" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q56" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R56" s="19" t="s">
+      <c r="P56" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q56" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R56" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -5760,16 +5760,16 @@
       <c r="N57" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="O57" s="19" t="s">
+      <c r="O57" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P57" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q57" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R57" s="19" t="s">
+      <c r="P57" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q57" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R57" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -5816,16 +5816,16 @@
       <c r="N58" s="4" t="s">
         <v>609</v>
       </c>
-      <c r="O58" s="19" t="s">
+      <c r="O58" s="16" t="s">
         <v>701</v>
       </c>
-      <c r="P58" s="19" t="s">
+      <c r="P58" s="16" t="s">
         <v>702</v>
       </c>
-      <c r="Q58" s="19" t="s">
+      <c r="Q58" s="16" t="s">
         <v>644</v>
       </c>
-      <c r="R58" s="19" t="s">
+      <c r="R58" s="16" t="s">
         <v>703</v>
       </c>
     </row>
@@ -5872,16 +5872,16 @@
       <c r="N59" s="4" t="s">
         <v>413</v>
       </c>
-      <c r="O59" s="19" t="s">
+      <c r="O59" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P59" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q59" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R59" s="19" t="s">
+      <c r="P59" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q59" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R59" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -5928,16 +5928,16 @@
       <c r="N60" s="4" t="s">
         <v>614</v>
       </c>
-      <c r="O60" s="19" t="s">
+      <c r="O60" s="16" t="s">
         <v>704</v>
       </c>
-      <c r="P60" s="19" t="s">
+      <c r="P60" s="16" t="s">
         <v>705</v>
       </c>
-      <c r="Q60" s="19" t="s">
+      <c r="Q60" s="16" t="s">
         <v>706</v>
       </c>
-      <c r="R60" s="19" t="s">
+      <c r="R60" s="16" t="s">
         <v>707</v>
       </c>
     </row>
@@ -5984,16 +5984,16 @@
       <c r="N61" s="4" t="s">
         <v>427</v>
       </c>
-      <c r="O61" s="19" t="s">
+      <c r="O61" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P61" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q61" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R61" s="19" t="s">
+      <c r="P61" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q61" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R61" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -6040,16 +6040,16 @@
       <c r="N62" s="4" t="s">
         <v>435</v>
       </c>
-      <c r="O62" s="19" t="s">
+      <c r="O62" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P62" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q62" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R62" s="19" t="s">
+      <c r="P62" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q62" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R62" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -6096,16 +6096,16 @@
       <c r="N63" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="O63" s="19" t="s">
+      <c r="O63" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P63" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q63" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R63" s="19" t="s">
+      <c r="P63" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q63" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R63" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -6152,16 +6152,16 @@
       <c r="N64" s="4" t="s">
         <v>448</v>
       </c>
-      <c r="O64" s="19" t="s">
+      <c r="O64" s="16" t="s">
         <v>708</v>
       </c>
-      <c r="P64" s="19" t="s">
+      <c r="P64" s="16" t="s">
         <v>709</v>
       </c>
-      <c r="Q64" s="19" t="s">
+      <c r="Q64" s="16" t="s">
         <v>710</v>
       </c>
-      <c r="R64" s="19" t="s">
+      <c r="R64" s="16" t="s">
         <v>711</v>
       </c>
     </row>
@@ -6208,16 +6208,16 @@
       <c r="N65" s="4" t="s">
         <v>456</v>
       </c>
-      <c r="O65" s="19" t="s">
+      <c r="O65" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P65" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q65" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R65" s="19" t="s">
+      <c r="P65" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q65" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R65" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -6264,16 +6264,16 @@
       <c r="N66" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="O66" s="19" t="s">
+      <c r="O66" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P66" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q66" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R66" s="19" t="s">
+      <c r="P66" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q66" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R66" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -6320,16 +6320,16 @@
       <c r="N67" s="4" t="s">
         <v>470</v>
       </c>
-      <c r="O67" s="19" t="s">
+      <c r="O67" s="16" t="s">
         <v>712</v>
       </c>
-      <c r="P67" s="19" t="s">
+      <c r="P67" s="16" t="s">
         <v>713</v>
       </c>
-      <c r="Q67" s="19" t="s">
+      <c r="Q67" s="16" t="s">
         <v>714</v>
       </c>
-      <c r="R67" s="19" t="s">
+      <c r="R67" s="16" t="s">
         <v>715</v>
       </c>
     </row>
@@ -6376,16 +6376,16 @@
       <c r="N68" s="4" t="s">
         <v>478</v>
       </c>
-      <c r="O68" s="19" t="s">
+      <c r="O68" s="16" t="s">
         <v>716</v>
       </c>
-      <c r="P68" s="19" t="s">
+      <c r="P68" s="16" t="s">
         <v>717</v>
       </c>
-      <c r="Q68" s="19" t="s">
+      <c r="Q68" s="16" t="s">
         <v>718</v>
       </c>
-      <c r="R68" s="19" t="s">
+      <c r="R68" s="16" t="s">
         <v>719</v>
       </c>
     </row>
@@ -6432,20 +6432,20 @@
       <c r="N69" s="4" t="s">
         <v>605</v>
       </c>
-      <c r="O69" s="19" t="s">
+      <c r="O69" s="16" t="s">
         <v>720</v>
       </c>
-      <c r="P69" s="19" t="s">
+      <c r="P69" s="16" t="s">
         <v>721</v>
       </c>
-      <c r="Q69" s="19" t="s">
+      <c r="Q69" s="16" t="s">
         <v>722</v>
       </c>
-      <c r="R69" s="19" t="s">
+      <c r="R69" s="16" t="s">
         <v>723</v>
       </c>
     </row>
-    <row r="70" spans="1:18" ht="72" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:18" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A70" s="3" t="s">
         <v>482</v>
       </c>
@@ -6488,17 +6488,17 @@
       <c r="N70" s="4" t="s">
         <v>470</v>
       </c>
-      <c r="O70" s="19" t="s">
+      <c r="O70" s="16" t="s">
+        <v>739</v>
+      </c>
+      <c r="P70" s="16" t="s">
         <v>724</v>
       </c>
-      <c r="P70" s="19" t="s">
+      <c r="Q70" s="16" t="s">
+        <v>740</v>
+      </c>
+      <c r="R70" s="16" t="s">
         <v>725</v>
-      </c>
-      <c r="Q70" s="19" t="s">
-        <v>726</v>
-      </c>
-      <c r="R70" s="19" t="s">
-        <v>727</v>
       </c>
     </row>
     <row r="71" spans="1:18" ht="86.4" x14ac:dyDescent="0.3">
@@ -6544,16 +6544,16 @@
       <c r="N71" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="O71" s="19" t="s">
+      <c r="O71" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P71" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q71" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R71" s="19" t="s">
+      <c r="P71" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q71" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R71" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -6600,17 +6600,17 @@
       <c r="N72" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="O72" s="19" t="s">
+      <c r="O72" s="16" t="s">
+        <v>726</v>
+      </c>
+      <c r="P72" s="16" t="s">
+        <v>727</v>
+      </c>
+      <c r="Q72" s="16" t="s">
         <v>728</v>
       </c>
-      <c r="P72" s="19" t="s">
+      <c r="R72" s="16" t="s">
         <v>729</v>
-      </c>
-      <c r="Q72" s="19" t="s">
-        <v>730</v>
-      </c>
-      <c r="R72" s="19" t="s">
-        <v>731</v>
       </c>
     </row>
     <row r="73" spans="1:18" ht="100.8" x14ac:dyDescent="0.3">
@@ -6656,17 +6656,17 @@
       <c r="N73" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="O73" s="19" t="s">
+      <c r="O73" s="16" t="s">
+        <v>730</v>
+      </c>
+      <c r="P73" s="16" t="s">
+        <v>731</v>
+      </c>
+      <c r="Q73" s="16" t="s">
         <v>732</v>
       </c>
-      <c r="P73" s="19" t="s">
+      <c r="R73" s="16" t="s">
         <v>733</v>
-      </c>
-      <c r="Q73" s="19" t="s">
-        <v>734</v>
-      </c>
-      <c r="R73" s="19" t="s">
-        <v>735</v>
       </c>
     </row>
     <row r="74" spans="1:18" ht="86.4" x14ac:dyDescent="0.3">
@@ -6712,16 +6712,16 @@
       <c r="N74" s="4" t="s">
         <v>516</v>
       </c>
-      <c r="O74" s="19" t="s">
+      <c r="O74" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P74" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q74" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R74" s="19" t="s">
+      <c r="P74" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q74" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R74" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -6768,17 +6768,17 @@
       <c r="N75" s="4" t="s">
         <v>524</v>
       </c>
-      <c r="O75" s="19" t="s">
+      <c r="O75" s="16" t="s">
+        <v>734</v>
+      </c>
+      <c r="P75" s="16" t="s">
+        <v>735</v>
+      </c>
+      <c r="Q75" s="16" t="s">
         <v>736</v>
       </c>
-      <c r="P75" s="19" t="s">
+      <c r="R75" s="16" t="s">
         <v>737</v>
-      </c>
-      <c r="Q75" s="19" t="s">
-        <v>738</v>
-      </c>
-      <c r="R75" s="19" t="s">
-        <v>739</v>
       </c>
     </row>
     <row r="76" spans="1:18" ht="86.4" x14ac:dyDescent="0.3">
@@ -6824,16 +6824,16 @@
       <c r="N76" s="4" t="s">
         <v>531</v>
       </c>
-      <c r="O76" s="19" t="s">
+      <c r="O76" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P76" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q76" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R76" s="19" t="s">
+      <c r="P76" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q76" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R76" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -6880,16 +6880,16 @@
       <c r="N77" s="4" t="s">
         <v>537</v>
       </c>
-      <c r="O77" s="19" t="s">
+      <c r="O77" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P77" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q77" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R77" s="19" t="s">
+      <c r="P77" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q77" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R77" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -6936,16 +6936,16 @@
       <c r="N78" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="O78" s="19" t="s">
+      <c r="O78" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P78" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q78" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R78" s="19" t="s">
+      <c r="P78" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q78" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R78" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -6992,16 +6992,16 @@
       <c r="N79" s="4" t="s">
         <v>470</v>
       </c>
-      <c r="O79" s="19" t="s">
+      <c r="O79" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P79" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q79" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R79" s="19" t="s">
+      <c r="P79" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q79" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R79" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -7048,16 +7048,16 @@
       <c r="N80" s="4" t="s">
         <v>557</v>
       </c>
-      <c r="O80" s="19" t="s">
+      <c r="O80" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P80" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q80" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R80" s="19" t="s">
+      <c r="P80" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q80" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R80" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -7104,16 +7104,16 @@
       <c r="N81" s="4" t="s">
         <v>566</v>
       </c>
-      <c r="O81" s="19" t="s">
+      <c r="O81" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P81" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q81" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R81" s="19" t="s">
+      <c r="P81" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q81" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R81" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -7160,16 +7160,16 @@
       <c r="N82" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="O82" s="19" t="s">
+      <c r="O82" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P82" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q82" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R82" s="19" t="s">
+      <c r="P82" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q82" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R82" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -7216,16 +7216,16 @@
       <c r="N83" s="4" t="s">
         <v>578</v>
       </c>
-      <c r="O83" s="19" t="s">
+      <c r="O83" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P83" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q83" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R83" s="19" t="s">
+      <c r="P83" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q83" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R83" s="16" t="s">
         <v>637</v>
       </c>
     </row>
@@ -7272,16 +7272,16 @@
       <c r="N84" s="4" t="s">
         <v>586</v>
       </c>
-      <c r="O84" s="19" t="s">
+      <c r="O84" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="P84" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="Q84" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="R84" s="19" t="s">
+      <c r="P84" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="Q84" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="R84" s="16" t="s">
         <v>637</v>
       </c>
     </row>

</xml_diff>